<commit_message>
style: match the tracker templates to the original sheet design
Rebuilds all three templates against the formatting of the personal
Blind 75 sheet rather than an approximation of it: Arial throughout, the
six-stat merged dashboard, the dark banner rows, pattern-tinted column,
difficulty-coloured Diff, muted time budget, and the Shaky/OK/Strong
dropdown with its red/amber/green conditional formatting.

Verified cell-by-cell against the original — fonts, fills, alignment,
number formats, merges, freeze pane, column widths and row heights all
match exactly.

Also switches the README to a Drive "File -> Make a copy" flow (links
still to fill in), renames the Link column to NeetCode to match, and
names every tab "Tracker" so config.yml works unchanged across lists.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/blind75-tracker.xlsx
+++ b/templates/blind75-tracker.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$7:$K$82</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,60 +19,110 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="18">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F2933"/>
       <sz val="16"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF6B7280"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F2933"/>
-      <sz val="14"/>
+      <color rgb="FF475569"/>
+      <sz val="20"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF2563EB"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFB91C1C"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFB45309"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF047857"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF059669"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="FF6B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF10B981"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF6B7280"/>
       <sz val="9"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F2933"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001E6F42"/>
-    </font>
-    <font>
-      <color rgb="001A56DB"/>
+      <name val="Arial"/>
+      <color rgb="FF2563EB"/>
+      <sz val="10"/>
       <u val="single"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="008A6100"/>
+      <color rgb="FFF59E0B"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="009B1C1C"/>
+      <color rgb="FFEF4444"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -83,36 +131,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF2F7"/>
+        <fgColor rgb="FF1F2937"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2933"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E3F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDF3DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE4E4"/>
+        <fgColor rgb="FFEEF2FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -120,100 +148,122 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="001F2933"/>
-      </left>
-      <right style="thin">
-        <color rgb="001F2933"/>
-      </right>
-      <top style="thin">
-        <color rgb="001F2933"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="001F2933"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D8DEE6"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D8DEE6"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D8DEE6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D8DEE6"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="FF991B1B"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="FF92400E"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF3C7"/>
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="FF065F46"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD1FAE5"/>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -575,23 +625,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="4.38" customWidth="1" min="1" max="1"/>
+    <col width="19.25" customWidth="1" min="2" max="2"/>
+    <col width="33.25" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="9.630000000000001" customWidth="1" min="6" max="6"/>
+    <col width="11.38" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="39.38" customWidth="1" min="10" max="10"/>
+    <col width="11.38" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="11.38" customWidth="1" min="12" max="12"/>
+    <col width="7.63" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="27.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Blind 75 — Tracker</t>
@@ -605,203 +657,185 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Total problems</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Cold ✓</t>
-        </is>
-      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>1wk done</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>3wk done</t>
+          <t>Solved (any confidence)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Shaky</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>🔴 Shaky</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
+          <t>🟡 OK</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Strong</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>% Strong</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="4">
         <f>75</f>
         <v/>
       </c>
-      <c r="B4" s="4">
-        <f>COUNTA($G$8:$G$82)</f>
+      <c r="C4" s="5">
+        <f>COUNTA(K8:K82)</f>
         <v/>
       </c>
-      <c r="C4" s="4">
-        <f>COUNTA($H$8:$H$82)</f>
+      <c r="E4" s="6">
+        <f>COUNTIF(K8:K82,"Shaky")</f>
         <v/>
       </c>
-      <c r="D4" s="4">
-        <f>COUNTA($I$8:$I$82)</f>
+      <c r="G4" s="7">
+        <f>COUNTIF(K8:K82,"OK")</f>
         <v/>
       </c>
-      <c r="E4" s="4">
-        <f>COUNTIF($K$8:$K$82,"Shaky")</f>
+      <c r="I4" s="8">
+        <f>COUNTIF(K8:K82,"Strong")</f>
         <v/>
       </c>
-      <c r="F4" s="4">
-        <f>COUNTIF($K$8:$K$82,"OK")</f>
+      <c r="K4" s="9">
+        <f>IF(COUNTA(K8:K82)=0,0,COUNTIF(K8:K82,"Strong")/75)</f>
         <v/>
       </c>
-      <c r="G4" s="4">
-        <f>COUNTIF($K$8:$K$82,"Strong")</f>
-        <v/>
-      </c>
-      <c r="H4" s="5">
-        <f>IF(COUNTA($K$8:$K$82)=0,0,COUNTIF($K$8:$K$82,"Strong")/75)</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>4-pass method per problem: (1) cold attempt, timeboxed — no hints. (2) read the editorial/video. (3) re-solve from scratch. (4) write the key insight + the pitfall that got you, in your own words.</t>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>4-pass method per problem: (1) cold attempt 15-25min  →  (2) watch NeetCode + read editorial  →  (3) re-implement from scratch  →  (4) write key insight + pitfall</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Spaced repetition: re-solve each problem ~1 week and ~3 weeks after the cold attempt. Log the date you actually did it in the review columns — those blanks are what the nagger yells at you about.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Spaced repetition: re-solve cold 1 week later, then 3 weeks later. Mark confidence after each session. Shaky problems get re-reviewed next week regardless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="31.5" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Diff</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Time Budget</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>NeetCode</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Cold ✓ (date)</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>1wk Review</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>3wk Review</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>Key Insight + Pitfall</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Contains Duplicate</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n"/>
-      <c r="I8" s="13" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="20" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Valid Anagram</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -819,59 +853,59 @@
       <c r="G9" s="18" t="n"/>
       <c r="H9" s="18" t="n"/>
       <c r="I9" s="18" t="n"/>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="14" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="20" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Two Sum</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="n">
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="20" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Group Anagrams</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -889,66 +923,66 @@
       <c r="G11" s="18" t="n"/>
       <c r="H11" s="18" t="n"/>
       <c r="I11" s="18" t="n"/>
-      <c r="J11" s="16" t="n"/>
-      <c r="K11" s="14" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n">
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="20" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Top K Frequent Elements</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="13" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="n">
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>Encode and Decode Strings</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>~60min first / ~8min review  (LeetCode Premium — use the NeetCode link)</t>
+          <t>~60min first / ~8min review</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -959,59 +993,59 @@
       <c r="G13" s="18" t="n"/>
       <c r="H13" s="18" t="n"/>
       <c r="I13" s="18" t="n"/>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n">
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="20" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Product of Array Except Self</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
-      <c r="I14" s="13" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="n"/>
+      <c r="H14" s="18" t="n"/>
+      <c r="I14" s="18" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="20" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Longest Consecutive Sequence</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1029,59 +1063,59 @@
       <c r="G15" s="18" t="n"/>
       <c r="H15" s="18" t="n"/>
       <c r="I15" s="18" t="n"/>
-      <c r="J15" s="16" t="n"/>
-      <c r="K15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n">
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="20" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Two Pointers</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Valid Palindrome</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="n"/>
-      <c r="H16" s="13" t="n"/>
-      <c r="I16" s="13" t="n"/>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="n">
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="18" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="20" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Two Pointers</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>3Sum</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1099,59 +1133,59 @@
       <c r="G17" s="18" t="n"/>
       <c r="H17" s="18" t="n"/>
       <c r="I17" s="18" t="n"/>
-      <c r="J17" s="16" t="n"/>
-      <c r="K17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n">
+      <c r="J17" s="19" t="n"/>
+      <c r="K17" s="20" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Two Pointers</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Container with Most Water</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="n"/>
-      <c r="H18" s="13" t="n"/>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="n">
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="18" t="n"/>
+      <c r="I18" s="18" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="20" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>Best Time to Buy and Sell Stock</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -1169,59 +1203,59 @@
       <c r="G19" s="18" t="n"/>
       <c r="H19" s="18" t="n"/>
       <c r="I19" s="18" t="n"/>
-      <c r="J19" s="16" t="n"/>
-      <c r="K19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n">
+      <c r="J19" s="19" t="n"/>
+      <c r="K19" s="20" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Longest Substring without Repeating Characters</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="n">
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="n"/>
+      <c r="H20" s="18" t="n"/>
+      <c r="I20" s="18" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="20" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Longest Repeating Character Replacement</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1239,59 +1273,59 @@
       <c r="G21" s="18" t="n"/>
       <c r="H21" s="18" t="n"/>
       <c r="I21" s="18" t="n"/>
-      <c r="J21" s="16" t="n"/>
-      <c r="K21" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="n">
+      <c r="J21" s="19" t="n"/>
+      <c r="K21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Minimum Window Substring</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>~75min first / ~12min review</t>
         </is>
       </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="n"/>
-      <c r="H22" s="13" t="n"/>
-      <c r="I22" s="13" t="n"/>
-      <c r="J22" s="11" t="n"/>
-      <c r="K22" s="8" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="n">
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="18" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="20" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Stack</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Valid Parentheses</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -1309,59 +1343,59 @@
       <c r="G23" s="18" t="n"/>
       <c r="H23" s="18" t="n"/>
       <c r="I23" s="18" t="n"/>
-      <c r="J23" s="16" t="n"/>
-      <c r="K23" s="14" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="n">
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="20" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Binary Search</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>Find Minimum in Rotated Sorted Array</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
-      <c r="I24" s="13" t="n"/>
-      <c r="J24" s="11" t="n"/>
-      <c r="K24" s="8" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="n">
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="n"/>
+      <c r="H24" s="18" t="n"/>
+      <c r="I24" s="18" t="n"/>
+      <c r="J24" s="19" t="n"/>
+      <c r="K24" s="20" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Binary Search</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>Search in Rotated Sorted Array</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1379,59 +1413,59 @@
       <c r="G25" s="18" t="n"/>
       <c r="H25" s="18" t="n"/>
       <c r="I25" s="18" t="n"/>
-      <c r="J25" s="16" t="n"/>
-      <c r="K25" s="14" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="n">
+      <c r="J25" s="19" t="n"/>
+      <c r="K25" s="20" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>Reverse Linked List</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G26" s="13" t="n"/>
-      <c r="H26" s="13" t="n"/>
-      <c r="I26" s="13" t="n"/>
-      <c r="J26" s="11" t="n"/>
-      <c r="K26" s="8" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="n">
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="18" t="n"/>
+      <c r="I26" s="18" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="20" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>Merge Two Sorted Lists</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -1449,59 +1483,59 @@
       <c r="G27" s="18" t="n"/>
       <c r="H27" s="18" t="n"/>
       <c r="I27" s="18" t="n"/>
-      <c r="J27" s="16" t="n"/>
-      <c r="K27" s="14" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="n">
+      <c r="J27" s="19" t="n"/>
+      <c r="K27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>Linked List Cycle</t>
         </is>
       </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="11" t="n"/>
-      <c r="K28" s="8" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="n">
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="n"/>
+      <c r="H28" s="18" t="n"/>
+      <c r="I28" s="18" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="20" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Reorder List</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1519,59 +1553,59 @@
       <c r="G29" s="18" t="n"/>
       <c r="H29" s="18" t="n"/>
       <c r="I29" s="18" t="n"/>
-      <c r="J29" s="16" t="n"/>
-      <c r="K29" s="14" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="n">
+      <c r="J29" s="19" t="n"/>
+      <c r="K29" s="20" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>Remove Nth Node from End of List</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="13" t="n"/>
-      <c r="J30" s="11" t="n"/>
-      <c r="K30" s="8" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="14" t="n">
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="19" t="n"/>
+      <c r="K30" s="20" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr">
         <is>
           <t>Merge K Sorted Lists</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -1589,59 +1623,59 @@
       <c r="G31" s="18" t="n"/>
       <c r="H31" s="18" t="n"/>
       <c r="I31" s="18" t="n"/>
-      <c r="J31" s="16" t="n"/>
-      <c r="K31" s="14" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="n">
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>Invert Binary Tree</t>
         </is>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D32" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="13" t="n"/>
-      <c r="J32" s="11" t="n"/>
-      <c r="K32" s="8" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="n">
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="18" t="n"/>
+      <c r="J32" s="19" t="n"/>
+      <c r="K32" s="20" t="n"/>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>Maximum Depth of Binary Tree</t>
         </is>
       </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -1659,59 +1693,59 @@
       <c r="G33" s="18" t="n"/>
       <c r="H33" s="18" t="n"/>
       <c r="I33" s="18" t="n"/>
-      <c r="J33" s="16" t="n"/>
-      <c r="K33" s="14" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="n">
+      <c r="J33" s="19" t="n"/>
+      <c r="K33" s="20" t="n"/>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>Same Tree</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E34" s="11" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
-      <c r="I34" s="13" t="n"/>
-      <c r="J34" s="11" t="n"/>
-      <c r="K34" s="8" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="14" t="n">
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="19" t="n"/>
+      <c r="K34" s="20" t="n"/>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>Subtree of Another Tree</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -1729,59 +1763,59 @@
       <c r="G35" s="18" t="n"/>
       <c r="H35" s="18" t="n"/>
       <c r="I35" s="18" t="n"/>
-      <c r="J35" s="16" t="n"/>
-      <c r="K35" s="14" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="n">
+      <c r="J35" s="19" t="n"/>
+      <c r="K35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
         <is>
           <t>Lowest Common Ancestor of a Binary Search Tree</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="n"/>
-      <c r="H36" s="13" t="n"/>
-      <c r="I36" s="13" t="n"/>
-      <c r="J36" s="11" t="n"/>
-      <c r="K36" s="8" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="14" t="n">
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="18" t="n"/>
+      <c r="J36" s="19" t="n"/>
+      <c r="K36" s="20" t="n"/>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr">
         <is>
           <t>Binary Tree Level Order Traversal</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1799,59 +1833,59 @@
       <c r="G37" s="18" t="n"/>
       <c r="H37" s="18" t="n"/>
       <c r="I37" s="18" t="n"/>
-      <c r="J37" s="16" t="n"/>
-      <c r="K37" s="14" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="n">
+      <c r="J37" s="19" t="n"/>
+      <c r="K37" s="20" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>Validate Binary Search Tree</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E38" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="n"/>
-      <c r="H38" s="13" t="n"/>
-      <c r="I38" s="13" t="n"/>
-      <c r="J38" s="11" t="n"/>
-      <c r="K38" s="8" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="14" t="n">
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="18" t="n"/>
+      <c r="I38" s="18" t="n"/>
+      <c r="J38" s="19" t="n"/>
+      <c r="K38" s="20" t="n"/>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C39" s="14" t="inlineStr">
         <is>
           <t>Kth Smallest Element in a BST</t>
         </is>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1869,59 +1903,59 @@
       <c r="G39" s="18" t="n"/>
       <c r="H39" s="18" t="n"/>
       <c r="I39" s="18" t="n"/>
-      <c r="J39" s="16" t="n"/>
-      <c r="K39" s="14" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="n">
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="20" t="n"/>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>Construct Binary Tree from Preorder and Inorder Traversal</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E40" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="n"/>
-      <c r="H40" s="13" t="n"/>
-      <c r="I40" s="13" t="n"/>
-      <c r="J40" s="11" t="n"/>
-      <c r="K40" s="8" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="14" t="n">
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G40" s="18" t="n"/>
+      <c r="H40" s="18" t="n"/>
+      <c r="I40" s="18" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="20" t="n"/>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="12" t="n">
         <v>34</v>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C41" s="14" t="inlineStr">
         <is>
           <t>Binary Tree Maximum Path Sum</t>
         </is>
       </c>
-      <c r="D41" s="20" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -1939,59 +1973,59 @@
       <c r="G41" s="18" t="n"/>
       <c r="H41" s="18" t="n"/>
       <c r="I41" s="18" t="n"/>
-      <c r="J41" s="16" t="n"/>
-      <c r="K41" s="14" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="n">
+      <c r="J41" s="19" t="n"/>
+      <c r="K41" s="20" t="n"/>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Trees</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>Serialize and Deserialize Binary Tree</t>
         </is>
       </c>
-      <c r="D42" s="20" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="E42" s="11" t="inlineStr">
+      <c r="E42" s="16" t="inlineStr">
         <is>
           <t>~75min first / ~12min review</t>
         </is>
       </c>
-      <c r="F42" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G42" s="13" t="n"/>
-      <c r="H42" s="13" t="n"/>
-      <c r="I42" s="13" t="n"/>
-      <c r="J42" s="11" t="n"/>
-      <c r="K42" s="8" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="14" t="n">
+      <c r="F42" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G42" s="18" t="n"/>
+      <c r="H42" s="18" t="n"/>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="19" t="n"/>
+      <c r="K42" s="20" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>Heap / Priority Queue</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
         <is>
           <t>Find Median from Data Stream</t>
         </is>
       </c>
-      <c r="D43" s="20" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
@@ -2009,59 +2043,59 @@
       <c r="G43" s="18" t="n"/>
       <c r="H43" s="18" t="n"/>
       <c r="I43" s="18" t="n"/>
-      <c r="J43" s="16" t="n"/>
-      <c r="K43" s="14" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n">
+      <c r="J43" s="19" t="n"/>
+      <c r="K43" s="20" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Backtracking</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>Combination Sum</t>
         </is>
       </c>
-      <c r="D44" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E44" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F44" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G44" s="13" t="n"/>
-      <c r="H44" s="13" t="n"/>
-      <c r="I44" s="13" t="n"/>
-      <c r="J44" s="11" t="n"/>
-      <c r="K44" s="8" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="14" t="n">
+      <c r="D44" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G44" s="18" t="n"/>
+      <c r="H44" s="18" t="n"/>
+      <c r="I44" s="18" t="n"/>
+      <c r="J44" s="19" t="n"/>
+      <c r="K44" s="20" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>Backtracking</t>
         </is>
       </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>Word Search</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D45" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2079,59 +2113,59 @@
       <c r="G45" s="18" t="n"/>
       <c r="H45" s="18" t="n"/>
       <c r="I45" s="18" t="n"/>
-      <c r="J45" s="16" t="n"/>
-      <c r="K45" s="14" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n">
+      <c r="J45" s="19" t="n"/>
+      <c r="K45" s="20" t="n"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="12" t="n">
         <v>39</v>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>Tries</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>Implement Trie Prefix Tree</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E46" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F46" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G46" s="13" t="n"/>
-      <c r="H46" s="13" t="n"/>
-      <c r="I46" s="13" t="n"/>
-      <c r="J46" s="11" t="n"/>
-      <c r="K46" s="8" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="14" t="n">
+      <c r="D46" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F46" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G46" s="18" t="n"/>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="18" t="n"/>
+      <c r="J46" s="19" t="n"/>
+      <c r="K46" s="20" t="n"/>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="B47" s="14" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>Tries</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
         <is>
           <t>Design Add and Search Words Data Structure</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D47" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2149,59 +2183,59 @@
       <c r="G47" s="18" t="n"/>
       <c r="H47" s="18" t="n"/>
       <c r="I47" s="18" t="n"/>
-      <c r="J47" s="16" t="n"/>
-      <c r="K47" s="14" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="n">
+      <c r="J47" s="19" t="n"/>
+      <c r="K47" s="20" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>Tries</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>Word Search II</t>
         </is>
       </c>
-      <c r="D48" s="20" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="E48" s="11" t="inlineStr">
+      <c r="E48" s="16" t="inlineStr">
         <is>
           <t>~75min first / ~12min review</t>
         </is>
       </c>
-      <c r="F48" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G48" s="13" t="n"/>
-      <c r="H48" s="13" t="n"/>
-      <c r="I48" s="13" t="n"/>
-      <c r="J48" s="11" t="n"/>
-      <c r="K48" s="8" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="14" t="n">
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G48" s="18" t="n"/>
+      <c r="H48" s="18" t="n"/>
+      <c r="I48" s="18" t="n"/>
+      <c r="J48" s="19" t="n"/>
+      <c r="K48" s="20" t="n"/>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B49" s="14" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>Graphs</t>
         </is>
       </c>
-      <c r="C49" s="15" t="inlineStr">
+      <c r="C49" s="14" t="inlineStr">
         <is>
           <t>Number of Islands</t>
         </is>
       </c>
-      <c r="D49" s="19" t="inlineStr">
+      <c r="D49" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2219,59 +2253,59 @@
       <c r="G49" s="18" t="n"/>
       <c r="H49" s="18" t="n"/>
       <c r="I49" s="18" t="n"/>
-      <c r="J49" s="16" t="n"/>
-      <c r="K49" s="14" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="n">
+      <c r="J49" s="19" t="n"/>
+      <c r="K49" s="20" t="n"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="12" t="n">
         <v>43</v>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="13" t="inlineStr">
         <is>
           <t>Graphs</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>Clone Graph</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E50" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F50" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="13" t="n"/>
-      <c r="J50" s="11" t="n"/>
-      <c r="K50" s="8" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="14" t="n">
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G50" s="18" t="n"/>
+      <c r="H50" s="18" t="n"/>
+      <c r="I50" s="18" t="n"/>
+      <c r="J50" s="19" t="n"/>
+      <c r="K50" s="20" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="B51" s="13" t="inlineStr">
         <is>
           <t>Graphs</t>
         </is>
       </c>
-      <c r="C51" s="15" t="inlineStr">
+      <c r="C51" s="14" t="inlineStr">
         <is>
           <t>Pacific Atlantic Water Flow</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D51" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2289,66 +2323,66 @@
       <c r="G51" s="18" t="n"/>
       <c r="H51" s="18" t="n"/>
       <c r="I51" s="18" t="n"/>
-      <c r="J51" s="16" t="n"/>
-      <c r="K51" s="14" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="n">
+      <c r="J51" s="19" t="n"/>
+      <c r="K51" s="20" t="n"/>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>Graphs</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
         <is>
           <t>Course Schedule</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E52" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F52" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
-      <c r="I52" s="13" t="n"/>
-      <c r="J52" s="11" t="n"/>
-      <c r="K52" s="8" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="14" t="n">
+      <c r="D52" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G52" s="18" t="n"/>
+      <c r="H52" s="18" t="n"/>
+      <c r="I52" s="18" t="n"/>
+      <c r="J52" s="19" t="n"/>
+      <c r="K52" s="20" t="n"/>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="B53" s="14" t="inlineStr">
+      <c r="B53" s="13" t="inlineStr">
         <is>
           <t>Graphs</t>
         </is>
       </c>
-      <c r="C53" s="15" t="inlineStr">
+      <c r="C53" s="14" t="inlineStr">
         <is>
           <t>Graph Valid Tree</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="D53" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>~60min first / ~8min review  (LeetCode Premium — use the NeetCode link)</t>
+          <t>~60min first / ~8min review</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr">
@@ -2359,66 +2393,66 @@
       <c r="G53" s="18" t="n"/>
       <c r="H53" s="18" t="n"/>
       <c r="I53" s="18" t="n"/>
-      <c r="J53" s="16" t="n"/>
-      <c r="K53" s="14" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="n">
+      <c r="J53" s="19" t="n"/>
+      <c r="K53" s="20" t="n"/>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>Graphs</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>Number of Connected Components in an Undirected Graph</t>
         </is>
       </c>
-      <c r="D54" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E54" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review  (LeetCode Premium — use the NeetCode link)</t>
-        </is>
-      </c>
-      <c r="F54" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G54" s="13" t="n"/>
-      <c r="H54" s="13" t="n"/>
-      <c r="I54" s="13" t="n"/>
-      <c r="J54" s="11" t="n"/>
-      <c r="K54" s="8" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="14" t="n">
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="n"/>
+      <c r="H54" s="18" t="n"/>
+      <c r="I54" s="18" t="n"/>
+      <c r="J54" s="19" t="n"/>
+      <c r="K54" s="20" t="n"/>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="B55" s="14" t="inlineStr">
+      <c r="B55" s="13" t="inlineStr">
         <is>
           <t>Advanced Graphs</t>
         </is>
       </c>
-      <c r="C55" s="15" t="inlineStr">
+      <c r="C55" s="14" t="inlineStr">
         <is>
           <t>Alien Dictionary</t>
         </is>
       </c>
-      <c r="D55" s="20" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>~75min first / ~12min review  (LeetCode Premium — use the NeetCode link)</t>
+          <t>~75min first / ~12min review</t>
         </is>
       </c>
       <c r="F55" s="17" t="inlineStr">
@@ -2429,59 +2463,59 @@
       <c r="G55" s="18" t="n"/>
       <c r="H55" s="18" t="n"/>
       <c r="I55" s="18" t="n"/>
-      <c r="J55" s="16" t="n"/>
-      <c r="K55" s="14" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="n">
+      <c r="J55" s="19" t="n"/>
+      <c r="K55" s="20" t="n"/>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="12" t="n">
         <v>49</v>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C56" s="14" t="inlineStr">
         <is>
           <t>Climbing Stairs</t>
         </is>
       </c>
-      <c r="D56" s="10" t="inlineStr">
+      <c r="D56" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E56" s="11" t="inlineStr">
+      <c r="E56" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F56" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G56" s="13" t="n"/>
-      <c r="H56" s="13" t="n"/>
-      <c r="I56" s="13" t="n"/>
-      <c r="J56" s="11" t="n"/>
-      <c r="K56" s="8" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="14" t="n">
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="n"/>
+      <c r="H56" s="18" t="n"/>
+      <c r="I56" s="18" t="n"/>
+      <c r="J56" s="19" t="n"/>
+      <c r="K56" s="20" t="n"/>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="C57" s="14" t="inlineStr">
         <is>
           <t>House Robber</t>
         </is>
       </c>
-      <c r="D57" s="19" t="inlineStr">
+      <c r="D57" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2499,59 +2533,59 @@
       <c r="G57" s="18" t="n"/>
       <c r="H57" s="18" t="n"/>
       <c r="I57" s="18" t="n"/>
-      <c r="J57" s="16" t="n"/>
-      <c r="K57" s="14" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="n">
+      <c r="J57" s="19" t="n"/>
+      <c r="K57" s="20" t="n"/>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="12" t="n">
         <v>51</v>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>House Robber II</t>
         </is>
       </c>
-      <c r="D58" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E58" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F58" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G58" s="13" t="n"/>
-      <c r="H58" s="13" t="n"/>
-      <c r="I58" s="13" t="n"/>
-      <c r="J58" s="11" t="n"/>
-      <c r="K58" s="8" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="14" t="n">
+      <c r="D58" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="n"/>
+      <c r="H58" s="18" t="n"/>
+      <c r="I58" s="18" t="n"/>
+      <c r="J58" s="19" t="n"/>
+      <c r="K58" s="20" t="n"/>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="12" t="n">
         <v>52</v>
       </c>
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B59" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
+      <c r="C59" s="14" t="inlineStr">
         <is>
           <t>Longest Palindromic Substring</t>
         </is>
       </c>
-      <c r="D59" s="19" t="inlineStr">
+      <c r="D59" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2569,59 +2603,59 @@
       <c r="G59" s="18" t="n"/>
       <c r="H59" s="18" t="n"/>
       <c r="I59" s="18" t="n"/>
-      <c r="J59" s="16" t="n"/>
-      <c r="K59" s="14" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="n">
+      <c r="J59" s="19" t="n"/>
+      <c r="K59" s="20" t="n"/>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>Palindromic Substrings</t>
         </is>
       </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E60" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F60" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G60" s="13" t="n"/>
-      <c r="H60" s="13" t="n"/>
-      <c r="I60" s="13" t="n"/>
-      <c r="J60" s="11" t="n"/>
-      <c r="K60" s="8" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="14" t="n">
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G60" s="18" t="n"/>
+      <c r="H60" s="18" t="n"/>
+      <c r="I60" s="18" t="n"/>
+      <c r="J60" s="19" t="n"/>
+      <c r="K60" s="20" t="n"/>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="12" t="n">
         <v>54</v>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C61" s="15" t="inlineStr">
+      <c r="C61" s="14" t="inlineStr">
         <is>
           <t>Decode Ways</t>
         </is>
       </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="D61" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2639,59 +2673,59 @@
       <c r="G61" s="18" t="n"/>
       <c r="H61" s="18" t="n"/>
       <c r="I61" s="18" t="n"/>
-      <c r="J61" s="16" t="n"/>
-      <c r="K61" s="14" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="n">
+      <c r="J61" s="19" t="n"/>
+      <c r="K61" s="20" t="n"/>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="12" t="n">
         <v>55</v>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C62" s="14" t="inlineStr">
         <is>
           <t>Coin Change</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E62" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F62" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G62" s="13" t="n"/>
-      <c r="H62" s="13" t="n"/>
-      <c r="I62" s="13" t="n"/>
-      <c r="J62" s="11" t="n"/>
-      <c r="K62" s="8" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="14" t="n">
+      <c r="D62" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F62" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="n"/>
+      <c r="H62" s="18" t="n"/>
+      <c r="I62" s="18" t="n"/>
+      <c r="J62" s="19" t="n"/>
+      <c r="K62" s="20" t="n"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C63" s="15" t="inlineStr">
+      <c r="C63" s="14" t="inlineStr">
         <is>
           <t>Maximum Product Subarray</t>
         </is>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D63" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2709,59 +2743,59 @@
       <c r="G63" s="18" t="n"/>
       <c r="H63" s="18" t="n"/>
       <c r="I63" s="18" t="n"/>
-      <c r="J63" s="16" t="n"/>
-      <c r="K63" s="14" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="n">
+      <c r="J63" s="19" t="n"/>
+      <c r="K63" s="20" t="n"/>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="12" t="n">
         <v>57</v>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C64" s="14" t="inlineStr">
         <is>
           <t>Word Break</t>
         </is>
       </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E64" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F64" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G64" s="13" t="n"/>
-      <c r="H64" s="13" t="n"/>
-      <c r="I64" s="13" t="n"/>
-      <c r="J64" s="11" t="n"/>
-      <c r="K64" s="8" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="14" t="n">
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F64" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="n"/>
+      <c r="H64" s="18" t="n"/>
+      <c r="I64" s="18" t="n"/>
+      <c r="J64" s="19" t="n"/>
+      <c r="K64" s="20" t="n"/>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="12" t="n">
         <v>58</v>
       </c>
-      <c r="B65" s="14" t="inlineStr">
+      <c r="B65" s="13" t="inlineStr">
         <is>
           <t>1-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C65" s="15" t="inlineStr">
+      <c r="C65" s="14" t="inlineStr">
         <is>
           <t>Longest Increasing Subsequence</t>
         </is>
       </c>
-      <c r="D65" s="19" t="inlineStr">
+      <c r="D65" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2779,59 +2813,59 @@
       <c r="G65" s="18" t="n"/>
       <c r="H65" s="18" t="n"/>
       <c r="I65" s="18" t="n"/>
-      <c r="J65" s="16" t="n"/>
-      <c r="K65" s="14" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="n">
+      <c r="J65" s="19" t="n"/>
+      <c r="K65" s="20" t="n"/>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="12" t="n">
         <v>59</v>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
         <is>
           <t>2-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>Unique Paths</t>
         </is>
       </c>
-      <c r="D66" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E66" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F66" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G66" s="13" t="n"/>
-      <c r="H66" s="13" t="n"/>
-      <c r="I66" s="13" t="n"/>
-      <c r="J66" s="11" t="n"/>
-      <c r="K66" s="8" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="14" t="n">
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F66" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G66" s="18" t="n"/>
+      <c r="H66" s="18" t="n"/>
+      <c r="I66" s="18" t="n"/>
+      <c r="J66" s="19" t="n"/>
+      <c r="K66" s="20" t="n"/>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B67" s="13" t="inlineStr">
         <is>
           <t>2-D Dynamic Programming</t>
         </is>
       </c>
-      <c r="C67" s="15" t="inlineStr">
+      <c r="C67" s="14" t="inlineStr">
         <is>
           <t>Longest Common Subsequence</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D67" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2849,59 +2883,59 @@
       <c r="G67" s="18" t="n"/>
       <c r="H67" s="18" t="n"/>
       <c r="I67" s="18" t="n"/>
-      <c r="J67" s="16" t="n"/>
-      <c r="K67" s="14" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="n">
+      <c r="J67" s="19" t="n"/>
+      <c r="K67" s="20" t="n"/>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" s="12" t="n">
         <v>61</v>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>Greedy</t>
         </is>
       </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="C68" s="14" t="inlineStr">
         <is>
           <t>Maximum Subarray</t>
         </is>
       </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E68" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F68" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G68" s="13" t="n"/>
-      <c r="H68" s="13" t="n"/>
-      <c r="I68" s="13" t="n"/>
-      <c r="J68" s="11" t="n"/>
-      <c r="K68" s="8" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="14" t="n">
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F68" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="n"/>
+      <c r="H68" s="18" t="n"/>
+      <c r="I68" s="18" t="n"/>
+      <c r="J68" s="19" t="n"/>
+      <c r="K68" s="20" t="n"/>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="12" t="n">
         <v>62</v>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B69" s="13" t="inlineStr">
         <is>
           <t>Greedy</t>
         </is>
       </c>
-      <c r="C69" s="15" t="inlineStr">
+      <c r="C69" s="14" t="inlineStr">
         <is>
           <t>Jump Game</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
+      <c r="D69" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2919,59 +2953,59 @@
       <c r="G69" s="18" t="n"/>
       <c r="H69" s="18" t="n"/>
       <c r="I69" s="18" t="n"/>
-      <c r="J69" s="16" t="n"/>
-      <c r="K69" s="14" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="n">
+      <c r="J69" s="19" t="n"/>
+      <c r="K69" s="20" t="n"/>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="12" t="n">
         <v>63</v>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B70" s="13" t="inlineStr">
         <is>
           <t>Intervals</t>
         </is>
       </c>
-      <c r="C70" s="9" t="inlineStr">
+      <c r="C70" s="14" t="inlineStr">
         <is>
           <t>Insert Interval</t>
         </is>
       </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E70" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F70" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G70" s="13" t="n"/>
-      <c r="H70" s="13" t="n"/>
-      <c r="I70" s="13" t="n"/>
-      <c r="J70" s="11" t="n"/>
-      <c r="K70" s="8" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="14" t="n">
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F70" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="n"/>
+      <c r="H70" s="18" t="n"/>
+      <c r="I70" s="18" t="n"/>
+      <c r="J70" s="19" t="n"/>
+      <c r="K70" s="20" t="n"/>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="12" t="n">
         <v>64</v>
       </c>
-      <c r="B71" s="14" t="inlineStr">
+      <c r="B71" s="13" t="inlineStr">
         <is>
           <t>Intervals</t>
         </is>
       </c>
-      <c r="C71" s="15" t="inlineStr">
+      <c r="C71" s="14" t="inlineStr">
         <is>
           <t>Merge Intervals</t>
         </is>
       </c>
-      <c r="D71" s="19" t="inlineStr">
+      <c r="D71" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2989,66 +3023,66 @@
       <c r="G71" s="18" t="n"/>
       <c r="H71" s="18" t="n"/>
       <c r="I71" s="18" t="n"/>
-      <c r="J71" s="16" t="n"/>
-      <c r="K71" s="14" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="n">
+      <c r="J71" s="19" t="n"/>
+      <c r="K71" s="20" t="n"/>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="12" t="n">
         <v>65</v>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>Intervals</t>
         </is>
       </c>
-      <c r="C72" s="9" t="inlineStr">
+      <c r="C72" s="14" t="inlineStr">
         <is>
           <t>Non Overlapping Intervals</t>
         </is>
       </c>
-      <c r="D72" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E72" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F72" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G72" s="13" t="n"/>
-      <c r="H72" s="13" t="n"/>
-      <c r="I72" s="13" t="n"/>
-      <c r="J72" s="11" t="n"/>
-      <c r="K72" s="8" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="14" t="n">
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="n"/>
+      <c r="H72" s="18" t="n"/>
+      <c r="I72" s="18" t="n"/>
+      <c r="J72" s="19" t="n"/>
+      <c r="K72" s="20" t="n"/>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="12" t="n">
         <v>66</v>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B73" s="13" t="inlineStr">
         <is>
           <t>Intervals</t>
         </is>
       </c>
-      <c r="C73" s="15" t="inlineStr">
+      <c r="C73" s="14" t="inlineStr">
         <is>
           <t>Meeting Rooms</t>
         </is>
       </c>
-      <c r="D73" s="10" t="inlineStr">
+      <c r="D73" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>~45min first / ~5min review  (LeetCode Premium — use the NeetCode link)</t>
+          <t>~45min first / ~5min review</t>
         </is>
       </c>
       <c r="F73" s="17" t="inlineStr">
@@ -3059,59 +3093,59 @@
       <c r="G73" s="18" t="n"/>
       <c r="H73" s="18" t="n"/>
       <c r="I73" s="18" t="n"/>
-      <c r="J73" s="16" t="n"/>
-      <c r="K73" s="14" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="n">
+      <c r="J73" s="19" t="n"/>
+      <c r="K73" s="20" t="n"/>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="12" t="n">
         <v>67</v>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>Intervals</t>
         </is>
       </c>
-      <c r="C74" s="9" t="inlineStr">
+      <c r="C74" s="14" t="inlineStr">
         <is>
           <t>Meeting Rooms II</t>
         </is>
       </c>
-      <c r="D74" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E74" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review  (LeetCode Premium — use the NeetCode link)</t>
-        </is>
-      </c>
-      <c r="F74" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G74" s="13" t="n"/>
-      <c r="H74" s="13" t="n"/>
-      <c r="I74" s="13" t="n"/>
-      <c r="J74" s="11" t="n"/>
-      <c r="K74" s="8" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="14" t="n">
+      <c r="D74" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F74" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="n"/>
+      <c r="H74" s="18" t="n"/>
+      <c r="I74" s="18" t="n"/>
+      <c r="J74" s="19" t="n"/>
+      <c r="K74" s="20" t="n"/>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="12" t="n">
         <v>68</v>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B75" s="13" t="inlineStr">
         <is>
           <t>Math &amp; Geometry</t>
         </is>
       </c>
-      <c r="C75" s="15" t="inlineStr">
+      <c r="C75" s="14" t="inlineStr">
         <is>
           <t>Rotate Image</t>
         </is>
       </c>
-      <c r="D75" s="19" t="inlineStr">
+      <c r="D75" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3129,59 +3163,59 @@
       <c r="G75" s="18" t="n"/>
       <c r="H75" s="18" t="n"/>
       <c r="I75" s="18" t="n"/>
-      <c r="J75" s="16" t="n"/>
-      <c r="K75" s="14" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="n">
+      <c r="J75" s="19" t="n"/>
+      <c r="K75" s="20" t="n"/>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="12" t="n">
         <v>69</v>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B76" s="13" t="inlineStr">
         <is>
           <t>Math &amp; Geometry</t>
         </is>
       </c>
-      <c r="C76" s="9" t="inlineStr">
+      <c r="C76" s="14" t="inlineStr">
         <is>
           <t>Spiral Matrix</t>
         </is>
       </c>
-      <c r="D76" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E76" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F76" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G76" s="13" t="n"/>
-      <c r="H76" s="13" t="n"/>
-      <c r="I76" s="13" t="n"/>
-      <c r="J76" s="11" t="n"/>
-      <c r="K76" s="8" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="14" t="n">
+      <c r="D76" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F76" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G76" s="18" t="n"/>
+      <c r="H76" s="18" t="n"/>
+      <c r="I76" s="18" t="n"/>
+      <c r="J76" s="19" t="n"/>
+      <c r="K76" s="20" t="n"/>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="12" t="n">
         <v>70</v>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B77" s="13" t="inlineStr">
         <is>
           <t>Math &amp; Geometry</t>
         </is>
       </c>
-      <c r="C77" s="15" t="inlineStr">
+      <c r="C77" s="14" t="inlineStr">
         <is>
           <t>Set Matrix Zeroes</t>
         </is>
       </c>
-      <c r="D77" s="19" t="inlineStr">
+      <c r="D77" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3199,59 +3233,59 @@
       <c r="G77" s="18" t="n"/>
       <c r="H77" s="18" t="n"/>
       <c r="I77" s="18" t="n"/>
-      <c r="J77" s="16" t="n"/>
-      <c r="K77" s="14" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="8" t="n">
+      <c r="J77" s="19" t="n"/>
+      <c r="K77" s="20" t="n"/>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="12" t="n">
         <v>71</v>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B78" s="13" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="C78" s="9" t="inlineStr">
+      <c r="C78" s="14" t="inlineStr">
         <is>
           <t>Number of 1 Bits</t>
         </is>
       </c>
-      <c r="D78" s="10" t="inlineStr">
+      <c r="D78" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E78" s="11" t="inlineStr">
+      <c r="E78" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F78" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G78" s="13" t="n"/>
-      <c r="H78" s="13" t="n"/>
-      <c r="I78" s="13" t="n"/>
-      <c r="J78" s="11" t="n"/>
-      <c r="K78" s="8" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="14" t="n">
+      <c r="F78" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G78" s="18" t="n"/>
+      <c r="H78" s="18" t="n"/>
+      <c r="I78" s="18" t="n"/>
+      <c r="J78" s="19" t="n"/>
+      <c r="K78" s="20" t="n"/>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="12" t="n">
         <v>72</v>
       </c>
-      <c r="B79" s="14" t="inlineStr">
+      <c r="B79" s="13" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="C79" s="15" t="inlineStr">
+      <c r="C79" s="14" t="inlineStr">
         <is>
           <t>Counting Bits</t>
         </is>
       </c>
-      <c r="D79" s="10" t="inlineStr">
+      <c r="D79" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -3269,59 +3303,59 @@
       <c r="G79" s="18" t="n"/>
       <c r="H79" s="18" t="n"/>
       <c r="I79" s="18" t="n"/>
-      <c r="J79" s="16" t="n"/>
-      <c r="K79" s="14" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="8" t="n">
+      <c r="J79" s="19" t="n"/>
+      <c r="K79" s="20" t="n"/>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="12" t="n">
         <v>73</v>
       </c>
-      <c r="B80" s="8" t="inlineStr">
+      <c r="B80" s="13" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="C80" s="9" t="inlineStr">
+      <c r="C80" s="14" t="inlineStr">
         <is>
           <t>Reverse Bits</t>
         </is>
       </c>
-      <c r="D80" s="10" t="inlineStr">
+      <c r="D80" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="E80" s="11" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>~45min first / ~5min review</t>
         </is>
       </c>
-      <c r="F80" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G80" s="13" t="n"/>
-      <c r="H80" s="13" t="n"/>
-      <c r="I80" s="13" t="n"/>
-      <c r="J80" s="11" t="n"/>
-      <c r="K80" s="8" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="14" t="n">
+      <c r="F80" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G80" s="18" t="n"/>
+      <c r="H80" s="18" t="n"/>
+      <c r="I80" s="18" t="n"/>
+      <c r="J80" s="19" t="n"/>
+      <c r="K80" s="20" t="n"/>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="12" t="n">
         <v>74</v>
       </c>
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B81" s="13" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="C81" s="15" t="inlineStr">
+      <c r="C81" s="14" t="inlineStr">
         <is>
           <t>Missing Number</t>
         </is>
       </c>
-      <c r="D81" s="10" t="inlineStr">
+      <c r="D81" s="15" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
@@ -3339,46 +3373,74 @@
       <c r="G81" s="18" t="n"/>
       <c r="H81" s="18" t="n"/>
       <c r="I81" s="18" t="n"/>
-      <c r="J81" s="16" t="n"/>
-      <c r="K81" s="14" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="8" t="n">
+      <c r="J81" s="19" t="n"/>
+      <c r="K81" s="20" t="n"/>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="13" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="C82" s="9" t="inlineStr">
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>Sum of Two Integers</t>
         </is>
       </c>
-      <c r="D82" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E82" s="11" t="inlineStr">
-        <is>
-          <t>~60min first / ~8min review</t>
-        </is>
-      </c>
-      <c r="F82" s="12" t="inlineStr">
-        <is>
-          <t>Open →</t>
-        </is>
-      </c>
-      <c r="G82" s="13" t="n"/>
-      <c r="H82" s="13" t="n"/>
-      <c r="I82" s="13" t="n"/>
-      <c r="J82" s="11" t="n"/>
-      <c r="K82" s="8" t="n"/>
+      <c r="D82" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>~60min first / ~8min review</t>
+        </is>
+      </c>
+      <c r="F82" s="17" t="inlineStr">
+        <is>
+          <t>Open →</t>
+        </is>
+      </c>
+      <c r="G82" s="18" t="n"/>
+      <c r="H82" s="18" t="n"/>
+      <c r="I82" s="18" t="n"/>
+      <c r="J82" s="19" t="n"/>
+      <c r="K82" s="20" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A7:K82"/>
+  <mergeCells count="16">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="C4:D4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="K8:K82">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Shaky"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Strong"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="K8:K82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Shaky,OK,Strong"</formula1>

</xml_diff>